<commit_message>
Added data set from Lamantia et al. (2026, Nature)
2000-year methane record from the Nevado Huascarán summit ice core.
</commit_message>
<xml_diff>
--- a/data/byrd-data-info.xlsx
+++ b/data/byrd-data-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\18596\Desktop\ByrdDIT_2026\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin Weber\AppData\Roaming\MathWorks\MATLAB Add-Ons\Collections\ByrdDIT - The Byrd Data Import Tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB8425C-C431-4662-91C8-B2A9A78497E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D868AA4-F77E-44A9-A223-BB6A307F5D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="368" windowWidth="21600" windowHeight="11054" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publication" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="131">
   <si>
     <t>bona-churchill</t>
   </si>
@@ -425,6 +425,12 @@
   </si>
   <si>
     <t>184TG-summary-concentrations</t>
+  </si>
+  <si>
+    <t>Lamantia et al. (2026)</t>
+  </si>
+  <si>
+    <t>summit-CH4</t>
   </si>
 </sst>
 </file>
@@ -743,28 +749,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{067D0BDD-F9FE-417B-A94C-024A55B5A08D}">
   <dimension ref="A1:S8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.86328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.53125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="19.86328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" customWidth="1"/>
-    <col min="19" max="19" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.86328125" customWidth="1"/>
+    <col min="19" max="19" width="18.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -823,7 +829,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -849,7 +855,7 @@
         <v>97</v>
       </c>
       <c r="I2" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="J2" t="s">
         <v>100</v>
@@ -882,7 +888,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -893,7 +899,7 @@
         <v>93</v>
       </c>
       <c r="I3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J3" t="s">
         <v>101</v>
@@ -905,7 +911,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
         <v>90</v>
       </c>
@@ -913,7 +919,7 @@
         <v>113</v>
       </c>
       <c r="I4" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="M4" t="s">
         <v>112</v>
@@ -922,25 +928,28 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
       <c r="F5" t="s">
         <v>114</v>
       </c>
       <c r="I5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
       <c r="F6" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="I6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
       <c r="F7" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
       <c r="F8" t="s">
         <v>95</v>
       </c>
@@ -952,44 +961,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF50EB8-00C0-4B81-9C39-E2A1C82D00CC}">
-  <dimension ref="A1:AJ11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AK11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.53125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.53125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="19.86328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="19.88671875" customWidth="1"/>
-    <col min="20" max="20" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.5546875" customWidth="1"/>
-    <col min="27" max="27" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="25.109375" customWidth="1"/>
-    <col min="36" max="36" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="19.86328125" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.53125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.53125" customWidth="1"/>
+    <col min="28" max="28" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="30.1328125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="21.796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="25.1328125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="25.1328125" customWidth="1"/>
+    <col min="37" max="37" width="18.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1054,19 +1063,19 @@
         <v>25</v>
       </c>
       <c r="V1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="W1" t="s">
         <v>36</v>
       </c>
       <c r="X1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y1" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>40</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>48</v>
       </c>
       <c r="AA1" t="s">
         <v>48</v>
@@ -1075,7 +1084,7 @@
         <v>48</v>
       </c>
       <c r="AC1" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="AD1" t="s">
         <v>56</v>
@@ -1084,22 +1093,25 @@
         <v>56</v>
       </c>
       <c r="AF1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AG1" t="s">
         <v>67</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>71</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>79</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>125</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -1152,64 +1164,67 @@
         <v>97</v>
       </c>
       <c r="R2" t="s">
+        <v>129</v>
+      </c>
+      <c r="S2" t="s">
         <v>118</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>123</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>98</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>99</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>101</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>100</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>116</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>102</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>121</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>103</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>112</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>105</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>106</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>104</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>107</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>108</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" t="s">
         <v>109</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AJ2" t="s">
         <v>126</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1262,64 +1277,67 @@
         <v>77</v>
       </c>
       <c r="R3" t="s">
+        <v>130</v>
+      </c>
+      <c r="S3" t="s">
         <v>119</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>124</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>35</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>26</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>38</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>37</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Y3" t="s">
         <v>1</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>41</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>122</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
         <v>8</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AC3" t="s">
         <v>49</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>60</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
         <v>63</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AF3" t="s">
         <v>57</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AG3" t="s">
         <v>68</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AH3" t="s">
         <v>1</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AI3" t="s">
         <v>80</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AJ3" t="s">
         <v>127</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AK3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1353,41 +1371,41 @@
       <c r="Q4" t="s">
         <v>6</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>120</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>27</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>42</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AB4" t="s">
         <v>55</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AC4" t="s">
         <v>50</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>61</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
         <v>62</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>58</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AG4" t="s">
         <v>69</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AI4" t="s">
         <v>81</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AJ4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.45">
       <c r="F5" t="s">
         <v>7</v>
       </c>
@@ -1403,91 +1421,91 @@
       <c r="Q5" t="s">
         <v>78</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>28</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>43</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AC5" t="s">
         <v>51</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>66</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AE5" t="s">
         <v>64</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>59</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AG5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.45">
       <c r="O6" t="s">
         <v>21</v>
       </c>
       <c r="Q6" t="s">
         <v>75</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>29</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>44</v>
       </c>
-      <c r="AB6" t="s">
+      <c r="AC6" t="s">
         <v>52</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AE6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.45">
       <c r="Q7" t="s">
         <v>74</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>30</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>45</v>
       </c>
-      <c r="AB7" t="s">
+      <c r="AC7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.45">
       <c r="Q8" t="s">
         <v>76</v>
       </c>
-      <c r="U8" t="s">
+      <c r="V8" t="s">
         <v>31</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Z8" t="s">
         <v>46</v>
       </c>
-      <c r="AB8" t="s">
+      <c r="AC8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="U9" t="s">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.45">
+      <c r="V9" t="s">
         <v>32</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="U10" t="s">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.45">
+      <c r="V10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="U11" t="s">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.45">
+      <c r="V11" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1499,29 +1517,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.53125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.53125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="31.6640625" customWidth="1"/>
     <col min="9" max="9" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.53125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.1328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.53125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1577,7 +1595,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1633,7 +1651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1674,7 +1692,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1703,7 +1721,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
         <v>8</v>
       </c>
@@ -1726,7 +1744,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
         <v>9</v>
       </c>
@@ -1749,7 +1767,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F7" t="s">
         <v>16</v>
       </c>
@@ -1769,7 +1787,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F8" t="s">
         <v>17</v>
       </c>
@@ -1786,7 +1804,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F9" t="s">
         <v>18</v>
       </c>
@@ -1800,7 +1818,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F10" t="s">
         <v>19</v>
       </c>
@@ -1811,7 +1829,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F11" t="s">
         <v>20</v>
       </c>
@@ -1822,32 +1840,32 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F15" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="F16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:6" x14ac:dyDescent="0.45">
       <c r="F17" t="s">
         <v>85</v>
       </c>

</xml_diff>